<commit_message>
Add per-region and across-region baseline x stim MLM analyses
- New v2 R scripts (run_v2_encoding.R, run_v2_retrieval.R) with per-region
  power/coherence models, across-region pooled models, and PAC models
  restricted to amygdala-target pairs (MTL: BLA-HPC/EC/PRC; HPC: BLA-HPC/CA/DG)
- Separate models for each frequency band to avoid multicollinearity
- Encoding: theta, slow gamma, HFA; Retrieval: theta, slow gamma only
- Balanced and imbalanced trial versions via --balanced/--imbalanced flags
- Unified report builder (build_v2_report.py) generates all 4 PDF reports
- Prior balanced/imbalanced MLM scripts and report builders preserved
- Various IED, hypothesis, and data processing scripts added

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/IED/AMMEBLAES_IEDs_trial_level_dissertation_test.xlsx
+++ b/IED/AMMEBLAES_IEDs_trial_level_dissertation_test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinahollearn/Library/CloudStorage/Box-Box/InmanLab/BLAES_data/dissertation/AMME_BLAES/IED/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{192011A0-13CB-0E4F-9DB6-52E381480CA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1610A85-DD1F-FB48-9172-CE9DA210A91B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="31680" yWindow="1320" windowWidth="29400" windowHeight="17280" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="580" windowWidth="29920" windowHeight="17620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -191,7 +191,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5698" uniqueCount="209">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5751" uniqueCount="209">
   <si>
     <t>Patient</t>
   </si>
@@ -21810,6 +21810,9 @@
       <c r="B617" t="s">
         <v>139</v>
       </c>
+      <c r="C617" t="s">
+        <v>130</v>
+      </c>
       <c r="D617" t="s">
         <v>22</v>
       </c>
@@ -21907,6 +21910,9 @@
       <c r="B620" t="s">
         <v>139</v>
       </c>
+      <c r="C620" t="s">
+        <v>130</v>
+      </c>
       <c r="D620" t="s">
         <v>22</v>
       </c>
@@ -22104,6 +22110,9 @@
       <c r="B626" t="s">
         <v>139</v>
       </c>
+      <c r="C626" t="s">
+        <v>130</v>
+      </c>
       <c r="D626" t="s">
         <v>22</v>
       </c>
@@ -22204,6 +22213,9 @@
       <c r="B629" t="s">
         <v>139</v>
       </c>
+      <c r="C629" t="s">
+        <v>130</v>
+      </c>
       <c r="D629" t="s">
         <v>22</v>
       </c>
@@ -22265,6 +22277,9 @@
       <c r="B631" t="s">
         <v>139</v>
       </c>
+      <c r="C631" t="s">
+        <v>130</v>
+      </c>
       <c r="D631" t="s">
         <v>22</v>
       </c>
@@ -22333,6 +22348,9 @@
       <c r="B633" t="s">
         <v>139</v>
       </c>
+      <c r="C633" t="s">
+        <v>130</v>
+      </c>
       <c r="D633" t="s">
         <v>22</v>
       </c>
@@ -22362,6 +22380,9 @@
       <c r="B634" t="s">
         <v>139</v>
       </c>
+      <c r="C634" t="s">
+        <v>130</v>
+      </c>
       <c r="D634" t="s">
         <v>22</v>
       </c>
@@ -22459,6 +22480,9 @@
       <c r="B637" t="s">
         <v>139</v>
       </c>
+      <c r="C637" t="s">
+        <v>130</v>
+      </c>
       <c r="D637" t="s">
         <v>22</v>
       </c>
@@ -22555,6 +22579,9 @@
       <c r="B640" t="s">
         <v>139</v>
       </c>
+      <c r="C640" t="s">
+        <v>130</v>
+      </c>
       <c r="D640" t="s">
         <v>22</v>
       </c>
@@ -22623,6 +22650,9 @@
       <c r="B642" t="s">
         <v>139</v>
       </c>
+      <c r="C642" t="s">
+        <v>130</v>
+      </c>
       <c r="D642" t="s">
         <v>22</v>
       </c>
@@ -22688,6 +22718,9 @@
       <c r="B644" t="s">
         <v>139</v>
       </c>
+      <c r="C644" t="s">
+        <v>130</v>
+      </c>
       <c r="D644" t="s">
         <v>22</v>
       </c>
@@ -22785,6 +22818,9 @@
       <c r="B647" t="s">
         <v>139</v>
       </c>
+      <c r="C647" t="s">
+        <v>130</v>
+      </c>
       <c r="D647" t="s">
         <v>22</v>
       </c>
@@ -22881,6 +22917,9 @@
       <c r="B650" t="s">
         <v>139</v>
       </c>
+      <c r="C650" t="s">
+        <v>130</v>
+      </c>
       <c r="D650" t="s">
         <v>22</v>
       </c>
@@ -22981,6 +23020,9 @@
       <c r="B653" t="s">
         <v>139</v>
       </c>
+      <c r="C653" t="s">
+        <v>130</v>
+      </c>
       <c r="D653" t="s">
         <v>22</v>
       </c>
@@ -23046,6 +23088,9 @@
       <c r="B655" t="s">
         <v>139</v>
       </c>
+      <c r="C655" t="s">
+        <v>130</v>
+      </c>
       <c r="D655" t="s">
         <v>22</v>
       </c>
@@ -23216,6 +23261,9 @@
       <c r="B660" t="s">
         <v>139</v>
       </c>
+      <c r="C660" t="s">
+        <v>130</v>
+      </c>
       <c r="D660" t="s">
         <v>22</v>
       </c>
@@ -23245,6 +23293,9 @@
       <c r="B661" t="s">
         <v>139</v>
       </c>
+      <c r="C661" t="s">
+        <v>130</v>
+      </c>
       <c r="D661" t="s">
         <v>22</v>
       </c>
@@ -23274,6 +23325,9 @@
       <c r="B662" t="s">
         <v>139</v>
       </c>
+      <c r="C662" t="s">
+        <v>130</v>
+      </c>
       <c r="D662" t="s">
         <v>22</v>
       </c>
@@ -23342,6 +23396,9 @@
       <c r="B664" t="s">
         <v>139</v>
       </c>
+      <c r="C664" t="s">
+        <v>130</v>
+      </c>
       <c r="D664" t="s">
         <v>22</v>
       </c>
@@ -23407,6 +23464,9 @@
       <c r="B666" t="s">
         <v>139</v>
       </c>
+      <c r="C666" t="s">
+        <v>130</v>
+      </c>
       <c r="D666" t="s">
         <v>22</v>
       </c>
@@ -23436,6 +23496,9 @@
       <c r="B667" t="s">
         <v>139</v>
       </c>
+      <c r="C667" t="s">
+        <v>130</v>
+      </c>
       <c r="D667" t="s">
         <v>22</v>
       </c>
@@ -23465,6 +23528,9 @@
       <c r="B668" t="s">
         <v>173</v>
       </c>
+      <c r="C668" t="s">
+        <v>130</v>
+      </c>
       <c r="D668" t="s">
         <v>22</v>
       </c>
@@ -23498,6 +23564,9 @@
       <c r="B669" t="s">
         <v>139</v>
       </c>
+      <c r="C669" t="s">
+        <v>130</v>
+      </c>
       <c r="D669" t="s">
         <v>22</v>
       </c>
@@ -23527,6 +23596,9 @@
       <c r="B670" t="s">
         <v>139</v>
       </c>
+      <c r="C670" t="s">
+        <v>130</v>
+      </c>
       <c r="D670" t="s">
         <v>22</v>
       </c>
@@ -23592,6 +23664,9 @@
       <c r="B672" t="s">
         <v>139</v>
       </c>
+      <c r="C672" t="s">
+        <v>130</v>
+      </c>
       <c r="D672" t="s">
         <v>22</v>
       </c>
@@ -23621,6 +23696,9 @@
       <c r="B673" t="s">
         <v>139</v>
       </c>
+      <c r="C673" t="s">
+        <v>130</v>
+      </c>
       <c r="D673" t="s">
         <v>22</v>
       </c>
@@ -23650,6 +23728,9 @@
       <c r="B674" t="s">
         <v>139</v>
       </c>
+      <c r="C674" t="s">
+        <v>130</v>
+      </c>
       <c r="D674" t="s">
         <v>22</v>
       </c>
@@ -23683,6 +23764,9 @@
       <c r="B675" t="s">
         <v>139</v>
       </c>
+      <c r="C675" t="s">
+        <v>130</v>
+      </c>
       <c r="D675" t="s">
         <v>22</v>
       </c>
@@ -23712,6 +23796,9 @@
       <c r="B676" t="s">
         <v>139</v>
       </c>
+      <c r="C676" t="s">
+        <v>130</v>
+      </c>
       <c r="D676" t="s">
         <v>22</v>
       </c>
@@ -23741,6 +23828,9 @@
       <c r="B677" t="s">
         <v>139</v>
       </c>
+      <c r="C677" t="s">
+        <v>130</v>
+      </c>
       <c r="D677" t="s">
         <v>22</v>
       </c>
@@ -23774,6 +23864,9 @@
       <c r="B678" t="s">
         <v>139</v>
       </c>
+      <c r="C678" t="s">
+        <v>130</v>
+      </c>
       <c r="D678" t="s">
         <v>22</v>
       </c>
@@ -23803,6 +23896,9 @@
       <c r="B679" t="s">
         <v>139</v>
       </c>
+      <c r="C679" t="s">
+        <v>130</v>
+      </c>
       <c r="D679" t="s">
         <v>22</v>
       </c>
@@ -23832,6 +23928,9 @@
       <c r="B680" t="s">
         <v>139</v>
       </c>
+      <c r="C680" t="s">
+        <v>130</v>
+      </c>
       <c r="D680" t="s">
         <v>22</v>
       </c>
@@ -23900,6 +23999,9 @@
       <c r="B682" t="s">
         <v>139</v>
       </c>
+      <c r="C682" t="s">
+        <v>130</v>
+      </c>
       <c r="D682" t="s">
         <v>22</v>
       </c>
@@ -23929,6 +24031,9 @@
       <c r="B683" t="s">
         <v>139</v>
       </c>
+      <c r="C683" t="s">
+        <v>130</v>
+      </c>
       <c r="D683" t="s">
         <v>22</v>
       </c>
@@ -23958,6 +24063,9 @@
       <c r="B684" t="s">
         <v>139</v>
       </c>
+      <c r="C684" t="s">
+        <v>130</v>
+      </c>
       <c r="D684" t="s">
         <v>22</v>
       </c>
@@ -23990,6 +24098,9 @@
       <c r="B685" t="s">
         <v>139</v>
       </c>
+      <c r="C685" t="s">
+        <v>130</v>
+      </c>
       <c r="D685" t="s">
         <v>22</v>
       </c>
@@ -24058,6 +24169,9 @@
       <c r="B687" t="s">
         <v>139</v>
       </c>
+      <c r="C687" t="s">
+        <v>130</v>
+      </c>
       <c r="D687" t="s">
         <v>22</v>
       </c>
@@ -24087,6 +24201,9 @@
       <c r="B688" t="s">
         <v>139</v>
       </c>
+      <c r="C688" t="s">
+        <v>130</v>
+      </c>
       <c r="D688" t="s">
         <v>22</v>
       </c>
@@ -24152,6 +24269,9 @@
       <c r="B690" t="s">
         <v>139</v>
       </c>
+      <c r="C690" t="s">
+        <v>130</v>
+      </c>
       <c r="D690" t="s">
         <v>22</v>
       </c>
@@ -24181,6 +24301,9 @@
       <c r="B691" t="s">
         <v>139</v>
       </c>
+      <c r="C691" t="s">
+        <v>130</v>
+      </c>
       <c r="D691" t="s">
         <v>22</v>
       </c>
@@ -24242,6 +24365,9 @@
       <c r="B693" t="s">
         <v>139</v>
       </c>
+      <c r="C693" t="s">
+        <v>130</v>
+      </c>
       <c r="D693" t="s">
         <v>22</v>
       </c>
@@ -24310,6 +24436,9 @@
       <c r="B695" t="s">
         <v>139</v>
       </c>
+      <c r="C695" t="s">
+        <v>130</v>
+      </c>
       <c r="D695" t="s">
         <v>22</v>
       </c>
@@ -24339,6 +24468,9 @@
       <c r="B696" t="s">
         <v>139</v>
       </c>
+      <c r="C696" t="s">
+        <v>130</v>
+      </c>
       <c r="D696" t="s">
         <v>22</v>
       </c>
@@ -24368,6 +24500,9 @@
       <c r="B697" t="s">
         <v>139</v>
       </c>
+      <c r="C697" t="s">
+        <v>130</v>
+      </c>
       <c r="D697" t="s">
         <v>22</v>
       </c>
@@ -24401,6 +24536,9 @@
       <c r="B698" t="s">
         <v>139</v>
       </c>
+      <c r="C698" t="s">
+        <v>130</v>
+      </c>
       <c r="D698" t="s">
         <v>22</v>
       </c>
@@ -24431,7 +24569,7 @@
         <v>192</v>
       </c>
       <c r="C699" t="s">
-        <v>193</v>
+        <v>130</v>
       </c>
       <c r="D699" t="s">
         <v>22</v>
@@ -24462,6 +24600,9 @@
       <c r="B700" t="s">
         <v>139</v>
       </c>
+      <c r="C700" t="s">
+        <v>130</v>
+      </c>
       <c r="D700" t="s">
         <v>22</v>
       </c>
@@ -24527,6 +24668,9 @@
       <c r="B702" t="s">
         <v>139</v>
       </c>
+      <c r="C702" t="s">
+        <v>130</v>
+      </c>
       <c r="D702" t="s">
         <v>15</v>
       </c>
@@ -24560,6 +24704,9 @@
       <c r="B703" t="s">
         <v>139</v>
       </c>
+      <c r="C703" t="s">
+        <v>130</v>
+      </c>
       <c r="D703" t="s">
         <v>15</v>
       </c>
@@ -24657,6 +24804,9 @@
       <c r="B706" t="s">
         <v>139</v>
       </c>
+      <c r="C706" t="s">
+        <v>130</v>
+      </c>
       <c r="D706" t="s">
         <v>22</v>
       </c>
@@ -24686,6 +24836,9 @@
       <c r="B707" t="s">
         <v>139</v>
       </c>
+      <c r="C707" t="s">
+        <v>130</v>
+      </c>
       <c r="D707" t="s">
         <v>15</v>
       </c>
@@ -24875,6 +25028,9 @@
       <c r="B713" t="s">
         <v>139</v>
       </c>
+      <c r="C713" t="s">
+        <v>130</v>
+      </c>
       <c r="D713" t="s">
         <v>22</v>
       </c>
@@ -24907,6 +25063,9 @@
       </c>
       <c r="B714" t="s">
         <v>139</v>
+      </c>
+      <c r="C714" t="s">
+        <v>130</v>
       </c>
       <c r="D714" t="s">
         <v>22</v>

</xml_diff>